<commit_message>
Enhance attorney verification with city detection, organization extraction, and frontend integration
</commit_message>
<xml_diff>
--- a/backend/data/verified/verified_attorneys.xlsx
+++ b/backend/data/verified/verified_attorneys.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,51 +413,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>s_no</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>reg_no</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>organization</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>page_title</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
         <is>
           <t>bio</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>source_url</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
@@ -494,29 +492,45 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>Rochester</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>tate.tischner@troutman.com</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>585.270.2109</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Tate uses his technical training and scientific research background to advise health sciences and agricultural clients on protecting and maximizing the value of their innovations.
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Tate L. Tischner - Troutman Pepper Locke</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tate uses his technical training and scientific research background to advise health sciences and agricultural clients on protecting and maximizing the value of their innovations.
+Troutman Pepper Locke’s National Intellectual Property Practice and 13 Attorneys Honored in IAM Patent 1000 2026
 Tate is the managing partner of the Rochester office and a registered patent attorney who counsels clients on domestic and foreign utility patent prosecution, plant patents, plant variety certificates, interferences, reexaminations, reissues, foreign oppositions, licensing, noninfringement and validity opinions, and patent litigation.
 He has handled legal matters in a variety of technologies, with particular emphasis in biotechnology, molecular biology, plants, agricultural technology, medicinal chemistry, synthetic chemistry, membrane technology, and medical devices.
 In the botanical and agricultural technology areas, Tate has broad experience in patent prosecution, plant patenting, and plant variety protection, for crops, ornamental plants, genetically modified plants, plant-breeding technologies, agricultural compositions, plant varieties, various food-related technologies (e.g., food compositions, health and functional foods, food additives, food-related products for treatment of human diseases, and animal feed compositions), farm equipment and implements, and opinions, patent disputes, and litigation for major crops.
-Tate has presented to numerous groups on topics related to intellectual property law, including diagnostic methods patents, plant protection, subject matter eligibility for biotech</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
+Tate has presented to numerous groups on topics related to intellectual property law, including diagnostic methods patents, plant protection, subject matter eligibility for biotechnology inventions, patent legislation, promulgation of new patent rules, Patent and Trademark Office procedures, patent prosecution strategies, and post-issuance procedures and strategies.
+His technical training is in biology, botany, agriculture, genetics, and organic chemistry. As a graduate student, he conducted and published research related to quantitative traits in soybean.
+Troutman Pepper Locke’s National Intellectual Property Practice and 13 Attorneys Honored in IAM Patent 1000 2026
+Tate is the managing partner of the Rochester office and a registered patent attorney who counsels clients on domestic and foreign utility patent prosecution, plant patents, plant variety certificates, interferences, reexaminations, reissues, foreign oppositions, licensing, noninfringement and validity opinions, and patent litigation.
+He has handled legal matters in a variety of technologies, with particular emphasis in biotechnology, molecular biology, plants, agricultural technology, medicinal chemistry, synthetic chemistry, membrane technology, and medical devices.
+</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>https://www.troutman.com/professionals/tate-l-tischner/</t>
         </is>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
         <v>100</v>
       </c>
     </row>
@@ -539,28 +553,42 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>peter.zhou@troutman.com</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>404.870.4688</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Dr. Zhou advises a variety of clients, including multinational corporations, international research institutes, startups, and independent inventors on the prosecution of utility and design patents as well as strategic patent portfolio development and management. He also provides clients with the counsel they need on a variety of matters, including non-infringement and/or invalidity analysis, design around, freedom-to-operate, and patentability.
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Peter Peng Zhou, Ph.D. - Troutman Pepper Locke</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dr. Zhou advises a variety of clients, including multinational corporations, international research institutes, startups, and independent inventors on the prosecution of utility and design patents as well as strategic patent portfolio development and management. He also provides clients with the counsel they need on a variety of matters, including non-infringement and/or invalidity analysis, design around, freedom-to-operate, and patentability.
 Dr. Zhou prosecutes patents in a broad array of technological fields, including biomedical engineering, medical physics and medical devices, life science, physics, nanotechnology, material science, telecommunications, fiber optics, photonics and electronics, quantum communications and computations, optical, mechanical and electronic devices, semiconductors, computer software, mass spectrometry, blockchain, and artificial intelligence.
 Before his career as a patent agent, Dr. Zhou served in engineering and research roles throughout the U.S., U.K., and the EU, where he focused on areas of technology such as laser physics, photonics and quantum electronics, fiber optics, optical networking, quantum computer, quantum communications, modeling of complex systems, computer-aided measurements and automations, data acquisition and signal conditioning, and micro-electrical-mechanical systems (MEMS).
-Dr. Zhou has published more than 80 research articles inPhysical Review Letters,Physical Review A, and other leading academic research journals. Add</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
+Dr. Zhou has published more than 80 research articles inPhysical Review Letters,Physical Review A, and other leading academic research journals. Additionally, Dr. Zhou had acted as referee for several leading academic research journals in physics and optics.
+Dr. Zhou advises a variety of clients, including multinational corporations, international research institutes, startups, and independent inventors on the prosecution of utility and design patents as well as strategic patent portfolio development and management. He also provides clients with the counsel they need on a variety of matters, including non-infringement and/or invalidity analysis, design around, freedom-to-operate, and patentability.
+Dr. Zhou prosecutes patents in a broad array of technological fields, including biomedical engineering, medical physics and medical devices, life science, physics, nanotechnology, material science, telecommunications, fiber optics, photonics and electronics, quantum communications and computations, optical, mechanical and electronic devices, semiconductors, computer software, mass spectrometry, blockchain, and artificial intelligence.
+Before his career as a patent agent, Dr. Zhou served in engineering and research roles throughout the U.S., U.K., and the EU, where he focused on areas of technology such as laser physics, photonics and quantum electronics, fiber optics, optical networking, quantum computer, quantum communications, modeling of complex systems, computer-aided measurements and automations, data acquisition and signal conditioning, and micro-electrical-mechanical systems (MEMS).
+</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>https://www.troutman.com/professionals/peter-peng-zhou-phd/</t>
         </is>
       </c>
-      <c r="I3" t="n">
+      <c r="K3" t="n">
         <v>100</v>
       </c>
     </row>
@@ -570,38 +598,56 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mark D Alleman</t>
+          <t>Mandy Song</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>42257</v>
+        <v>69583</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Alleman Hall LLP</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>mark@allemanhall.com</t>
-        </is>
-      </c>
+          <t>Bayes PLLC</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>503.595.7300</t>
+          <t>mandy.song@bayes.law</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mark D. Alleman - Alleman Hall LLP | Patent &amp; Trademark Law Firm About Us Team Services Contact Careers EN JP @ 2026 ALLEMAN HALL CREASMAN &amp; TUTTLE LLP Mark D. Alleman Partner Portland Office email mark@allemanhall.com tel 503.595.7300 Education Degrees J.D., University of Oregon (Order of the Coif) (1998) Japanese Ministry of Education Research Student, Kyoto Institute of Technology (1994-95) B.S., Engineering (Product Design), Stanford University (1993) Career Professional Highlights Mark D. Alleman represents clients in all aspects of patent and trademark matters, including patentability studies, non-infringement and invalidity studies, due diligence, preparation and prosecution of patent and trademark applications before the USPTO, licensing and litigation. Mark works with companies large and small engaged in technical fields such as computer software and hardware, computer networking, augmented and virtual reality, wearable computing, computer operating systems, machine learning, data center optimization, gaming consoles, mobile telephones, printers, heavy equipment, automobiles, motorcycles, off-road utility vehicles, personal watercraft, thin films, semiconductor manufacturing, mass flow controllers, precision measurement and test equipment, radar and sonar equipment, and toys. Mark is active in both the firm’s domestic and international practices. Mark speaks Japanese, travels to Japan frequently to lecture, and was previously admitted as a licensed foreign lawyer in </t>
+          <t>Not Found</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://allemanhall.com/person/mark-d-alleman/</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
+          <t>Mandy Song – Bayes PLLC</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cross-Border Disputes Between China and the United States: Litigation, Arbitration, and Enforcement
+Mega Verdicts in U.S. Patent Litigation: Willful Infringement, Exceptionality &amp; PTAB Challenges
+A New Era of Patent Practice and Litigation in Europe—The EU Unitary Patent and Unified Patent Court Brexit
+Opportunity to Get Your Application Allowed After Final Rejection—Introducing the After Final Consideration Pilot
+Workshop on Strategic Use of Administrative Invalidity Proceedings in Patent Litigation
+Bayes PLLC and its managing partner Mandy Song have recently completed the Minority Firm Incubator hosted by Harrity &amp; Harrity, LLP! The Minority Firm Incubator 2.0 is a 42-week program that provides the training and tools needed to propel female and minority-owned...
+On October 21, 2016, a massive and sustained Internet attack, specifically a distributed denial of service (DDOS) attack, caused network outages across large swaths of the United States and Europe. The attack launched with the...
+As part of Strafford Publications’ webinar series, Bayes partner Mandy Song was joined by Justin Cassell, Shareholder at Workman Nydegger, to discuss USPTO options for responding after final rejection of a patent application. The program reviewed the basics of each...
+The Internet of Things (IoT) is rapidly emerging to connect all objects around the world. You might ask what is special about that, we have been connecting things to the Internet for decades. The difference is the anticipated scale of connectivity and the intelligence...
+I. History of AFCP In the United States, after a final rejection is issued on a pending patent application, prosecution of the application is considered “closed,” and the applicant is generally not entitled to further consideration of any additional submission unless...
+Mandy Song, Ph.D. brings nearly 20 years’ experience in patent practice, including patent prosecution, client counseling, patent portfolio management &amp; transactions, patent litigation in U.S. federal district courts and Section 337 investigations at the U.S. International Trade Commission (ITC), and post-grant proceedings before the Patent Trial and Appeal Board (PTAB) of the U.S. Patent and Trademark Office (USPTO). She has significant experience in a wide range of electrical, computer, and biomedical technologies.
+Mandy is a seasoned attorney on patent office practice. She manages the development of large patent portfolios for more than 100 clients. She has personally drafted, filed, and prosecuted thousands of patent applications before the USPTO. She routinely interviews inventors to develop invention disclosures, drafts new patent applications in a broad range of complex technologies, conducts interviews with patent examiners, and appeals final rejections to the PTAB.
+</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://bayes.law/team-member/mandy-song/</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
         <v>100</v>
       </c>
     </row>
@@ -611,38 +657,238 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Matt Hall</t>
+          <t>John Kozlowski</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>43653</v>
+        <v>82124</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Alleman Hall LLP</t>
+          <t>Cooley LLP</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>matt@allemanhall.com</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>503.595.7300</t>
+          <t>jkozlowski@cooley.com</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Matt Hall - Alleman Hall LLP | Patent &amp; Trademark Law Firm About Us Team Services Contact Careers EN JP @ 2026 ALLEMAN HALL CREASMAN &amp; TUTTLE LLP Matt Hall Partner Portland Office email matt@allemanhall.com tel 503.595.7300 Education Degrees J.D., University of Colorado School of Law, Boulder, Colorado Ph.D., Inorganic Chemistry, Oregon State University, Corvallis, Oregon B.S., Chemistry, Wake Forest University, Winston-Salem, North Carolina Career Professional Highlights Matt Hall represents clients in a variety of intellectual property areas, including patentability studies, patent prosecution, patent invalidity, and non-infringement studies, patent licensing and litigation, and trademark prosecution. Has drafted and prosecuted patent applications in diverse technical fields, including electronic materials processing, semiconductor device fabrication, battery recycling and remanufacturing, fuel cell chemistry and design, emissions control systems, polymer chemistry, engineered wood products, digital and analog circuits, image data compression and processing systems, computer software and hardware, quantum computing network and Internet-related technologies, and optics. Prior to attending law school, performed research on the synthesis of thin films and bulk quantities of novel oxides for use as low dielectric constant materials in superconducting integrated circuit applications. Associations Belongs To Admitted to practice in the State of Oregon Registered to practice befor</t>
+          <t>650 843 5337</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://allemanhall.com/person/m-matthews-hall-ph-d/</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
+          <t>Dr. Johnny Kozlowski - Patent Agent // Cooley // Global Law Firm</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Johnny focuses his practice on patent prosecution, counseling and diligence for chemistry and life sciences clients. Leveraging his unique combination of technical experience in both natural and computer sciences, Johnny works with clients to prosecute domestic and foreign patents at the forefront of interdisciplinary innovation.
+This content is provided for general informational purposes only, and your access or use of the content does not create an attorney-client relationship between you or your organization and Cooley LLP, Cooley (UK) LLP, or any other affiliated practice or entity (collectively referred to as "Cooley"). By accessing this content, you agree that the information provided does not constitute legal or other professional advice. This content is not a substitute for obtaining legal advice from a qualified attorney licensed in your jurisdiction, and you should not act or refrain from acting based on this content. This content may be changed without notice. It is not guaranteed to be complete, correct or up to date, and it may not reflect the most current legal developments. Prior results do not guarantee a similar outcome. Do not send any confidential information to Cooley, as we do not have any duty to keep any information you provide to us confidential. When advising companies, our attorney-client relationship is with the company, not with any individual. This content may have been generated with the assistance of artificial intelligence (Al) in accordance with our Al Principles, may be considered Attorney Advertising and is subject to ourlegal notices.
+When you visit any website, it may store or retrieve information on your browser, mostly in the form of cookies. This information might be about you, your preferences or your device and is mostly used to make the site work as you expect it to. The information does not usually directly identify you, but it can give you a more personalized web experience. Because we respect your right to privacy, you can choose not to allow some types of cookies. Click on the different category headings to find out more and change our default settings. However, blocking some types of cookies may impact your experience of the site and the services we are able to offer.
+You may update your consent in this Cookie preference center at any time.View our cookie policy.View our legal notices.
+Strictly necessary cookies are essential to provide you with the services you request on our website and for our compliance under data protection law. They are usually set in response to actions taken by you which amount to a request for services, such as setting your preferences or filling in forms. You cannot opt out of these cookies. This type of cookie does not collect any personally identifiable information about you and does not track your browsing habits.
+</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://www.cooley.com/people/johnny-kozlowski</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Tamera M Weisser</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>47856</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Jones Day</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>858.314.1181</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Tamera M. Weisser Ph.D. | Lawyers | Jones Day</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Named an "IP Trailblazer" byThe National Law Journal, Dr. Tamera (Tammy) Weisser is leader of Jones Day's global patent prosecution group and has more than 25 years of experience in global patent portfolio development, management, and enforcement in biotechnology, particularly in the areas of antibodies, cell therapies, gene therapies, and diagnostics. Her practice also includes performing patent validity and freedom-to-operate analyses and conducting due diligence of patent portfolios for clients, including potential investors, acquirers, and licensees.
+On behalf of BioMarin, she established a worldwide patent portfolio for Palynziq®, an FDA-approved enzyme replacement therapy for phenylketonuria treatment. On behalf of NGM Biopharmaceuticals, Tammy coordinates the global patent strategy concerning aldafermin in clinical trials for the treatment of nonalcoholic steatohepatitis (NASH), as well as the therapeutic antibodies NGM707, NGM831, and NGM438 for the treatment of cancers and tumors. She has developed IP strategies for dozens of antibody therapeutics for clients, including AbbVie, Astellas/Agensys, BMS/Celgene, Kyowa Kirin, Merck &amp; Co., and Xencor. Commercial products for which Tammy has experience include Carvykti®, Embosphere®, Humira®, Kynamro®, Otezla®, Palynziq®, Pomalyst®, Revlimid®, and Synagis®.
+In addition, Tammy has in-depth experience ininter partesreview (IPR) proceedings. For example, she successfully defended AbbVie in two IPRs brought by Amgen, five IPRs brought by Coherus, and another IPR brought by Sandoz in connection with patents related to formulations for AbbVie's antibody adalimumab, marketed as Humira®, in which the PTAB denied institution of each petition.
+Most recently, Tammy served on the board of governors of BIOCOM, and she is consistently recognized as a top lawyer and for her leadership and contribution within the community.
+San Diego Business Journal: Women of Influence in Law (2025); Women of Influence — 50 Over 50 (2024)
+The Daily Journal: Top Women Lawyers in California (2017, 2018, 2020, 2021); Top Intellectual Property Lawyers in California (2018-2019)
+We use cookies to enhance site navigation, analyze site usage, and assist in our marketing efforts.  For more information on our use of cookies and your personal data, please review the “Cookie Details” by clicking on “Manage Cookie Settings” and review ourPrivacy Policy. By accepting the "Accept All Cookies" you agree to the storing of performance, functional and targeting cookies on your device as further detailed in the “Manage Cookie Settings”. Individual cookie choices can be selected in the “Manage Cookie Settings” and accepted by clicking on “Confirm My Choices”. If you do not agree to the storing of any cookies that are not strictly necessary for the functioning of the site on your device, click on “Reject All Cookies”.
+</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://www.jonesday.com/en/lawyers/w/tamera-weisser</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Tova Werblowsky</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>82311</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Jones Day</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>212.326.3791</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Tova Werblowsky Ph.D. | Lawyers | Jones Day</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dr. Tova Werblowsky focuses on prosecuting patent applications and representing clients in Patent Office proceedings such asinter partesreview (IPR) proceedings. She also has experience providing intellectual property due diligence services such as landscape and freedom to operate analyses in the pharmaceutical, biotech, chemical, and materials industries to clients such as POSCO-Future M, Merck, BioMarin Pharmaceuticals, and British American Tobacco.
+Prior to joining Jones Day, Tova was a professor of chemistry and physics at Touro University in New York City. She taught advanced seminars in nanoscience, computational chemistry, materials, and biomedical topics in addition to general chemistry and physics courses.
+Her graduate and postdoctoral research was in the application of computational methods to determine and predict the energies and structures of monolayer adsorption of organic materials on semi-metallic surfaces. She worked in collaboration with an experimental group in the area of surface microscopy to understand the unique images produced in these techniques and adapted computational techniques to the study of the interface of the 3D solid and the single-layer adsorbed molecules.
+Tova has coauthored several peer-reviewed scientific publications, including publications inThe Journal of Physical Chemistryand theProceedings of the National Academy of Sciences(PNAS).
+2009Solvent Effects on the Self-Assembly of 1-Bromoeicosane on Graphite. Part I.
+Scanning Tunneling Microscopy,J. Phys. Chem.C 11
+2009Solvent Effects on the Self-Assembly of 1-Bromoeicosane on Graphite. Part II. Theory,J. Phys. Chem. C113
+2008Chain-length effects on the self-assembly of short 1-bromoalkane and n-alkane monolayers on graphite,J. Phys. Chem. C
+2008Thermodynamical Equilibrium of Binary Supramolecular
+Networks at the Liquid−Solid Interface,J. Am. Chem. Soc 130
+June 2007An Experimental and Theoretical Study of the Formation of Nanostructures of
+Self-Assembled Cyanuric Acid through Hydrogen Bond Networks on
+Graphite,Journal of Physical Chemistry B 111
+November 2006Frustrated Ostwald ripening in self-assembled monolayers of
+cruciform pi-systems,Langmuir 22
+August 2005Toward Nanoscale Charge Transfer: Experimental and
+Theoretical Characterization of Self-Assembled Monolayers,Abstracts of Papers of The
+American Chemical Society 230
+April 2005Scanning Tunneling Microscopy and Theoretical Studies of 1-Halohexane Monolayers on Graphite: Functional Group Interactions,
+Self-Assembly, and Image Contrast,Proceedings of the National Academy of Sciences
+102
+</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://www.jonesday.com/en/lawyers/w/tova-werblowsky</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>John J Williams</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>63016</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Jones Day</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>ocamina@susmangodfrey.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(713) 651-9366</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Ophelia F. Camiña | Susman Godfrey L.L.P.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Few trial lawyers have obtained this level of victory for their clients.  And, she is just as successful in representing defendants.  For one client, who was sued for over $1 Billion, Ms. Camiña obtained not only a “take nothing” award, but also an award of her client’s attorney’s fees. ***
+Clients describe Ms. Camiña as “smart, gutsy and tenacious” and as having “the whole trial-lawyer package: confidence, competitiveness and good judgment.”
+Ms. Camiña’s trial practice includes complex commercial cases in state court, federal court and in arbitration.  She has represented plaintiffs and defendants in a broad array of commercial disputes.  Because of her extraordinary track record, she is especially sought by clients facing complex, high-stakes and “bet-the-company” cases.
+***These are just examples of completed cases, not a prediction of future outcomes.
+</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>https://www.susmangodfrey.com/attorneys/ophelia-f-camina/</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>